<commit_message>
FIX AF for ROR
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_zAK_fixes.xlsx
+++ b/SuppXLS/Scen_zAK_fixes.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="8710"/>
+    <workbookView windowWidth="18350" windowHeight="8710" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="INS" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet8" sheetId="8" r:id="rId2"/>
     <sheet name="Sheet9" sheetId="9" r:id="rId3"/>
+    <sheet name="ROR_has_no_regulation_cap" sheetId="10" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -127,8 +128,40 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>xli9</author>
+  </authors>
+  <commentList>
+    <comment ref="H9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>xli9:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+dam hydropower should also have some limits, bcz not all dam hydropower are TGR</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>~TFM_UPD</t>
   </si>
@@ -194,6 +227,39 @@
   </si>
   <si>
     <t>DELIV</t>
+  </si>
+  <si>
+    <t>*COM_FR is worse than utilization rate for ROR, but we need to put this constraint to avoild regulation capacities</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>attribute</t>
+  </si>
+  <si>
+    <t>PSET_SET</t>
+  </si>
+  <si>
+    <t>PSET_CI</t>
+  </si>
+  <si>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>ELE</t>
+  </si>
+  <si>
+    <t>ELCHYD</t>
+  </si>
+  <si>
+    <t>*HYD-DAM*</t>
+  </si>
+  <si>
+    <t>*HYD-ROR*</t>
   </si>
 </sst>
 </file>
@@ -206,13 +272,19 @@
     <numFmt numFmtId="176" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* \-??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.2"/>
+      <color rgb="FF212529"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -370,9 +442,11 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -380,13 +454,24 @@
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -688,7 +773,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
@@ -705,55 +790,52 @@
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -768,80 +850,86 @@
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="51">
+  <cellStyles count="52">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -893,6 +981,7 @@
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal 10" xfId="49"/>
     <cellStyle name="Normale_Scen_UC_IND-StrucConst" xfId="50"/>
+    <cellStyle name="Input 2" xfId="51"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1371,7 +1460,7 @@
       <c r="E21" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21" s="3">
         <v>0.5</v>
       </c>
       <c r="G21" t="str">
@@ -1406,4 +1495,94 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A3:K11"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="25.0909090909091" customWidth="1"/>
+    <col min="2" max="2" width="28.7272727272727" customWidth="1"/>
+    <col min="5" max="5" width="12.8181818181818" customWidth="1"/>
+    <col min="7" max="7" width="13.2727272727273" customWidth="1"/>
+    <col min="9" max="9" width="12.4545454545455" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:11">
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" ht="16" spans="1:11">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10">
+        <v>0.48</v>
+      </c>
+      <c r="I10"/>
+      <c r="J10"/>
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="K11" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>